<commit_message>
kazoh : - 맵 보상 추가
</commit_message>
<xml_diff>
--- a/30_table/01_테스트버전/Table_Data_Map.xlsx
+++ b/30_table/01_테스트버전/Table_Data_Map.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1447" uniqueCount="692">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1561" uniqueCount="692">
   <si>
     <t>작업자</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -11899,6 +11899,9 @@
       <c r="Q82" s="34">
         <v>0</v>
       </c>
+      <c r="R82" s="36" t="s">
+        <v>235</v>
+      </c>
     </row>
     <row r="83" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A83" s="36">
@@ -11954,6 +11957,9 @@
       <c r="Q83" s="34">
         <v>0</v>
       </c>
+      <c r="R83" s="36" t="s">
+        <v>235</v>
+      </c>
     </row>
     <row r="84" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A84" s="36">
@@ -12009,6 +12015,15 @@
       <c r="Q84" s="34">
         <v>0</v>
       </c>
+      <c r="R84" s="36" t="s">
+        <v>235</v>
+      </c>
+      <c r="U84" s="36" t="s">
+        <v>236</v>
+      </c>
+      <c r="V84" s="36" t="s">
+        <v>237</v>
+      </c>
     </row>
     <row r="85" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A85" s="36">
@@ -12064,6 +12079,9 @@
       <c r="Q85" s="34">
         <v>0</v>
       </c>
+      <c r="R85" s="36" t="s">
+        <v>235</v>
+      </c>
     </row>
     <row r="86" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A86" s="36">
@@ -12119,6 +12137,15 @@
       <c r="Q86" s="34">
         <v>0</v>
       </c>
+      <c r="R86" s="36" t="s">
+        <v>235</v>
+      </c>
+      <c r="U86" s="36" t="s">
+        <v>236</v>
+      </c>
+      <c r="V86" s="36" t="s">
+        <v>237</v>
+      </c>
     </row>
     <row r="87" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A87" s="36">
@@ -12174,6 +12201,9 @@
       <c r="Q87" s="34">
         <v>0</v>
       </c>
+      <c r="R87" s="36" t="s">
+        <v>235</v>
+      </c>
     </row>
     <row r="88" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A88" s="36">
@@ -12229,6 +12259,9 @@
       <c r="Q88" s="34">
         <v>0</v>
       </c>
+      <c r="R88" s="36" t="s">
+        <v>235</v>
+      </c>
     </row>
     <row r="89" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A89" s="36">
@@ -12284,6 +12317,15 @@
       <c r="Q89" s="34">
         <v>0</v>
       </c>
+      <c r="R89" s="36" t="s">
+        <v>235</v>
+      </c>
+      <c r="U89" s="36" t="s">
+        <v>236</v>
+      </c>
+      <c r="V89" s="36" t="s">
+        <v>237</v>
+      </c>
     </row>
     <row r="90" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A90" s="36">
@@ -12339,6 +12381,9 @@
       <c r="Q90" s="34">
         <v>0</v>
       </c>
+      <c r="R90" s="36" t="s">
+        <v>235</v>
+      </c>
     </row>
     <row r="91" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A91" s="36">
@@ -12394,6 +12439,15 @@
       <c r="Q91" s="34">
         <v>0</v>
       </c>
+      <c r="R91" s="36" t="s">
+        <v>235</v>
+      </c>
+      <c r="U91" s="36" t="s">
+        <v>236</v>
+      </c>
+      <c r="V91" s="36" t="s">
+        <v>237</v>
+      </c>
     </row>
     <row r="92" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A92" s="36">
@@ -12449,6 +12503,15 @@
       <c r="Q92" s="34">
         <v>0</v>
       </c>
+      <c r="R92" s="36" t="s">
+        <v>235</v>
+      </c>
+      <c r="U92" s="36" t="s">
+        <v>236</v>
+      </c>
+      <c r="V92" s="36" t="s">
+        <v>237</v>
+      </c>
     </row>
     <row r="93" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A93" s="36">
@@ -12504,6 +12567,15 @@
       <c r="Q93" s="34">
         <v>0</v>
       </c>
+      <c r="R93" s="36" t="s">
+        <v>235</v>
+      </c>
+      <c r="U93" s="36" t="s">
+        <v>236</v>
+      </c>
+      <c r="V93" s="36" t="s">
+        <v>237</v>
+      </c>
     </row>
     <row r="94" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A94" s="36">
@@ -12559,6 +12631,9 @@
       <c r="Q94" s="34">
         <v>0</v>
       </c>
+      <c r="R94" s="36" t="s">
+        <v>235</v>
+      </c>
     </row>
     <row r="95" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A95" s="36">
@@ -12614,6 +12689,15 @@
       <c r="Q95" s="34">
         <v>0</v>
       </c>
+      <c r="R95" s="36" t="s">
+        <v>235</v>
+      </c>
+      <c r="U95" s="36" t="s">
+        <v>236</v>
+      </c>
+      <c r="V95" s="36" t="s">
+        <v>237</v>
+      </c>
     </row>
     <row r="96" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A96" s="36">
@@ -12669,8 +12753,11 @@
       <c r="Q96" s="34">
         <v>0</v>
       </c>
-    </row>
-    <row r="97" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="R96" s="36" t="s">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="97" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A97" s="36">
         <v>50095</v>
       </c>
@@ -12724,8 +12811,17 @@
       <c r="Q97" s="34">
         <v>0</v>
       </c>
-    </row>
-    <row r="98" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="R97" s="36" t="s">
+        <v>235</v>
+      </c>
+      <c r="U97" s="36" t="s">
+        <v>236</v>
+      </c>
+      <c r="V97" s="36" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="98" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A98" s="36">
         <v>50096</v>
       </c>
@@ -12779,8 +12875,11 @@
       <c r="Q98" s="34">
         <v>0</v>
       </c>
-    </row>
-    <row r="99" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="R98" s="36" t="s">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="99" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A99" s="36">
         <v>50097</v>
       </c>
@@ -12834,8 +12933,11 @@
       <c r="Q99" s="34">
         <v>0</v>
       </c>
-    </row>
-    <row r="100" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="R99" s="36" t="s">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="100" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A100" s="36">
         <v>50098</v>
       </c>
@@ -12889,8 +12991,17 @@
       <c r="Q100" s="34">
         <v>0</v>
       </c>
-    </row>
-    <row r="101" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="R100" s="36" t="s">
+        <v>235</v>
+      </c>
+      <c r="U100" s="36" t="s">
+        <v>236</v>
+      </c>
+      <c r="V100" s="36" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="101" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A101" s="36">
         <v>50099</v>
       </c>
@@ -12944,8 +13055,11 @@
       <c r="Q101" s="34">
         <v>0</v>
       </c>
-    </row>
-    <row r="102" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="R101" s="36" t="s">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="102" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A102" s="36">
         <v>50100</v>
       </c>
@@ -12999,8 +13113,11 @@
       <c r="Q102" s="34">
         <v>0</v>
       </c>
-    </row>
-    <row r="103" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="R102" s="36" t="s">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="103" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A103" s="36">
         <v>50101</v>
       </c>
@@ -13054,8 +13171,11 @@
       <c r="Q103" s="34">
         <v>0</v>
       </c>
-    </row>
-    <row r="104" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="R103" s="36" t="s">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="104" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A104" s="36">
         <v>50102</v>
       </c>
@@ -13109,8 +13229,11 @@
       <c r="Q104" s="34">
         <v>0</v>
       </c>
-    </row>
-    <row r="105" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="R104" s="36" t="s">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="105" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A105" s="36">
         <v>50103</v>
       </c>
@@ -13164,8 +13287,17 @@
       <c r="Q105" s="34">
         <v>0</v>
       </c>
-    </row>
-    <row r="106" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="R105" s="36" t="s">
+        <v>235</v>
+      </c>
+      <c r="U105" s="36" t="s">
+        <v>236</v>
+      </c>
+      <c r="V105" s="36" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="106" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A106" s="36">
         <v>50104</v>
       </c>
@@ -13219,8 +13351,11 @@
       <c r="Q106" s="34">
         <v>0</v>
       </c>
-    </row>
-    <row r="107" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="R106" s="36" t="s">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="107" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A107" s="36">
         <v>50105</v>
       </c>
@@ -13274,8 +13409,17 @@
       <c r="Q107" s="34">
         <v>0</v>
       </c>
-    </row>
-    <row r="108" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="R107" s="36" t="s">
+        <v>235</v>
+      </c>
+      <c r="U107" s="36" t="s">
+        <v>236</v>
+      </c>
+      <c r="V107" s="36" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="108" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A108" s="36">
         <v>50106</v>
       </c>
@@ -13329,8 +13473,17 @@
       <c r="Q108" s="34">
         <v>0</v>
       </c>
-    </row>
-    <row r="109" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="R108" s="36" t="s">
+        <v>235</v>
+      </c>
+      <c r="U108" s="36" t="s">
+        <v>236</v>
+      </c>
+      <c r="V108" s="36" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="109" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A109" s="36">
         <v>50107</v>
       </c>
@@ -13384,8 +13537,11 @@
       <c r="Q109" s="34">
         <v>0</v>
       </c>
-    </row>
-    <row r="110" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="R109" s="36" t="s">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="110" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A110" s="36">
         <v>50108</v>
       </c>
@@ -13439,8 +13595,11 @@
       <c r="Q110" s="34">
         <v>0</v>
       </c>
-    </row>
-    <row r="111" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="R110" s="36" t="s">
+        <v>456</v>
+      </c>
+    </row>
+    <row r="111" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A111" s="36">
         <v>50109</v>
       </c>
@@ -13494,8 +13653,17 @@
       <c r="Q111" s="34">
         <v>0</v>
       </c>
-    </row>
-    <row r="112" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="R111" s="36" t="s">
+        <v>456</v>
+      </c>
+      <c r="U111" s="34" t="s">
+        <v>457</v>
+      </c>
+      <c r="V111" s="34" t="s">
+        <v>458</v>
+      </c>
+    </row>
+    <row r="112" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A112" s="36">
         <v>50110</v>
       </c>
@@ -13549,8 +13717,17 @@
       <c r="Q112" s="34">
         <v>0</v>
       </c>
-    </row>
-    <row r="113" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="R112" s="36" t="s">
+        <v>456</v>
+      </c>
+      <c r="U112" s="34" t="s">
+        <v>457</v>
+      </c>
+      <c r="V112" s="34" t="s">
+        <v>458</v>
+      </c>
+    </row>
+    <row r="113" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A113" s="36">
         <v>50111</v>
       </c>
@@ -13604,8 +13781,17 @@
       <c r="Q113" s="34">
         <v>0</v>
       </c>
-    </row>
-    <row r="114" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="R113" s="36" t="s">
+        <v>456</v>
+      </c>
+      <c r="U113" s="34" t="s">
+        <v>457</v>
+      </c>
+      <c r="V113" s="34" t="s">
+        <v>458</v>
+      </c>
+    </row>
+    <row r="114" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A114" s="36">
         <v>50112</v>
       </c>
@@ -13659,8 +13845,17 @@
       <c r="Q114" s="34">
         <v>0</v>
       </c>
-    </row>
-    <row r="115" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="R114" s="36" t="s">
+        <v>456</v>
+      </c>
+      <c r="U114" s="34" t="s">
+        <v>457</v>
+      </c>
+      <c r="V114" s="34" t="s">
+        <v>458</v>
+      </c>
+    </row>
+    <row r="115" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A115" s="36">
         <v>50113</v>
       </c>
@@ -13714,8 +13909,11 @@
       <c r="Q115" s="34">
         <v>0</v>
       </c>
-    </row>
-    <row r="116" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="R115" s="36" t="s">
+        <v>456</v>
+      </c>
+    </row>
+    <row r="116" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A116" s="36">
         <v>50114</v>
       </c>
@@ -13769,8 +13967,17 @@
       <c r="Q116" s="34">
         <v>0</v>
       </c>
-    </row>
-    <row r="117" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="R116" s="36" t="s">
+        <v>456</v>
+      </c>
+      <c r="U116" s="34" t="s">
+        <v>457</v>
+      </c>
+      <c r="V116" s="34" t="s">
+        <v>458</v>
+      </c>
+    </row>
+    <row r="117" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A117" s="36">
         <v>50115</v>
       </c>
@@ -13824,8 +14031,11 @@
       <c r="Q117" s="34">
         <v>0</v>
       </c>
-    </row>
-    <row r="118" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="R117" s="36" t="s">
+        <v>456</v>
+      </c>
+    </row>
+    <row r="118" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A118" s="36">
         <v>50116</v>
       </c>
@@ -13879,8 +14089,11 @@
       <c r="Q118" s="34">
         <v>0</v>
       </c>
-    </row>
-    <row r="119" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="R118" s="36" t="s">
+        <v>456</v>
+      </c>
+    </row>
+    <row r="119" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A119" s="36">
         <v>50117</v>
       </c>
@@ -13934,8 +14147,17 @@
       <c r="Q119" s="34">
         <v>0</v>
       </c>
-    </row>
-    <row r="120" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="R119" s="36" t="s">
+        <v>456</v>
+      </c>
+      <c r="U119" s="34" t="s">
+        <v>457</v>
+      </c>
+      <c r="V119" s="34" t="s">
+        <v>458</v>
+      </c>
+    </row>
+    <row r="120" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A120" s="36">
         <v>50118</v>
       </c>
@@ -13989,8 +14211,11 @@
       <c r="Q120" s="34">
         <v>0</v>
       </c>
-    </row>
-    <row r="121" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="R120" s="36" t="s">
+        <v>456</v>
+      </c>
+    </row>
+    <row r="121" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A121" s="36">
         <v>50119</v>
       </c>
@@ -14044,8 +14269,11 @@
       <c r="Q121" s="34">
         <v>0</v>
       </c>
-    </row>
-    <row r="122" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="R121" s="36" t="s">
+        <v>456</v>
+      </c>
+    </row>
+    <row r="122" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A122" s="36">
         <v>50120</v>
       </c>
@@ -14099,8 +14327,17 @@
       <c r="Q122" s="34">
         <v>0</v>
       </c>
-    </row>
-    <row r="123" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="R122" s="36" t="s">
+        <v>456</v>
+      </c>
+      <c r="U122" s="34" t="s">
+        <v>457</v>
+      </c>
+      <c r="V122" s="34" t="s">
+        <v>458</v>
+      </c>
+    </row>
+    <row r="123" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A123" s="36">
         <v>50121</v>
       </c>
@@ -14154,8 +14391,11 @@
       <c r="Q123" s="34">
         <v>0</v>
       </c>
-    </row>
-    <row r="124" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="R123" s="36" t="s">
+        <v>456</v>
+      </c>
+    </row>
+    <row r="124" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A124" s="36">
         <v>50122</v>
       </c>
@@ -14209,8 +14449,11 @@
       <c r="Q124" s="34">
         <v>0</v>
       </c>
-    </row>
-    <row r="125" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="R124" s="36" t="s">
+        <v>456</v>
+      </c>
+    </row>
+    <row r="125" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A125" s="36">
         <v>50123</v>
       </c>
@@ -14264,8 +14507,17 @@
       <c r="Q125" s="34">
         <v>0</v>
       </c>
-    </row>
-    <row r="126" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="R125" s="36" t="s">
+        <v>456</v>
+      </c>
+      <c r="U125" s="34" t="s">
+        <v>457</v>
+      </c>
+      <c r="V125" s="34" t="s">
+        <v>458</v>
+      </c>
+    </row>
+    <row r="126" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A126" s="36">
         <v>50124</v>
       </c>
@@ -14319,8 +14571,17 @@
       <c r="Q126" s="34">
         <v>0</v>
       </c>
-    </row>
-    <row r="127" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="R126" s="36" t="s">
+        <v>456</v>
+      </c>
+      <c r="U126" s="34" t="s">
+        <v>457</v>
+      </c>
+      <c r="V126" s="34" t="s">
+        <v>458</v>
+      </c>
+    </row>
+    <row r="127" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A127" s="36">
         <v>50125</v>
       </c>
@@ -14374,8 +14635,17 @@
       <c r="Q127" s="34">
         <v>0</v>
       </c>
-    </row>
-    <row r="128" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="R127" s="36" t="s">
+        <v>456</v>
+      </c>
+      <c r="U127" s="34" t="s">
+        <v>457</v>
+      </c>
+      <c r="V127" s="34" t="s">
+        <v>458</v>
+      </c>
+    </row>
+    <row r="128" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A128" s="36">
         <v>50126</v>
       </c>
@@ -14429,8 +14699,11 @@
       <c r="Q128" s="34">
         <v>0</v>
       </c>
-    </row>
-    <row r="129" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="R128" s="36" t="s">
+        <v>456</v>
+      </c>
+    </row>
+    <row r="129" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A129" s="36">
         <v>50127</v>
       </c>
@@ -14484,8 +14757,11 @@
       <c r="Q129" s="34">
         <v>0</v>
       </c>
-    </row>
-    <row r="130" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="R129" s="36" t="s">
+        <v>456</v>
+      </c>
+    </row>
+    <row r="130" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A130" s="36">
         <v>50128</v>
       </c>
@@ -14539,8 +14815,17 @@
       <c r="Q130" s="34">
         <v>0</v>
       </c>
-    </row>
-    <row r="131" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="R130" s="36" t="s">
+        <v>456</v>
+      </c>
+      <c r="U130" s="34" t="s">
+        <v>457</v>
+      </c>
+      <c r="V130" s="34" t="s">
+        <v>458</v>
+      </c>
+    </row>
+    <row r="131" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A131" s="36">
         <v>50129</v>
       </c>
@@ -14594,8 +14879,11 @@
       <c r="Q131" s="34">
         <v>0</v>
       </c>
-    </row>
-    <row r="132" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="R131" s="36" t="s">
+        <v>456</v>
+      </c>
+    </row>
+    <row r="132" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A132" s="36">
         <v>50130</v>
       </c>
@@ -14649,8 +14937,11 @@
       <c r="Q132" s="34">
         <v>0</v>
       </c>
-    </row>
-    <row r="133" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="R132" s="36" t="s">
+        <v>456</v>
+      </c>
+    </row>
+    <row r="133" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A133" s="36">
         <v>50131</v>
       </c>
@@ -14704,8 +14995,17 @@
       <c r="Q133" s="34">
         <v>0</v>
       </c>
-    </row>
-    <row r="134" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="R133" s="36" t="s">
+        <v>456</v>
+      </c>
+      <c r="U133" s="34" t="s">
+        <v>457</v>
+      </c>
+      <c r="V133" s="34" t="s">
+        <v>458</v>
+      </c>
+    </row>
+    <row r="134" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A134" s="36">
         <v>50132</v>
       </c>
@@ -14759,8 +15059,17 @@
       <c r="Q134" s="34">
         <v>0</v>
       </c>
-    </row>
-    <row r="135" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="R134" s="36" t="s">
+        <v>456</v>
+      </c>
+      <c r="U134" s="34" t="s">
+        <v>457</v>
+      </c>
+      <c r="V134" s="34" t="s">
+        <v>458</v>
+      </c>
+    </row>
+    <row r="135" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A135" s="36">
         <v>50133</v>
       </c>
@@ -14814,8 +15123,17 @@
       <c r="Q135" s="34">
         <v>0</v>
       </c>
-    </row>
-    <row r="136" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="R135" s="36" t="s">
+        <v>456</v>
+      </c>
+      <c r="U135" s="34" t="s">
+        <v>457</v>
+      </c>
+      <c r="V135" s="34" t="s">
+        <v>458</v>
+      </c>
+    </row>
+    <row r="136" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A136" s="36">
         <v>50134</v>
       </c>
@@ -14869,8 +15187,11 @@
       <c r="Q136" s="34">
         <v>0</v>
       </c>
-    </row>
-    <row r="137" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="R136" s="36" t="s">
+        <v>456</v>
+      </c>
+    </row>
+    <row r="137" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A137" s="36">
         <v>50135</v>
       </c>
@@ -14924,8 +15245,17 @@
       <c r="Q137" s="34">
         <v>0</v>
       </c>
-    </row>
-    <row r="138" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="R137" s="36" t="s">
+        <v>456</v>
+      </c>
+      <c r="U137" s="34" t="s">
+        <v>457</v>
+      </c>
+      <c r="V137" s="34" t="s">
+        <v>458</v>
+      </c>
+    </row>
+    <row r="138" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A138" s="36">
         <v>50136</v>
       </c>
@@ -14979,8 +15309,17 @@
       <c r="Q138" s="34">
         <v>0</v>
       </c>
-    </row>
-    <row r="139" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="R138" s="36" t="s">
+        <v>456</v>
+      </c>
+      <c r="U138" s="34" t="s">
+        <v>457</v>
+      </c>
+      <c r="V138" s="34" t="s">
+        <v>458</v>
+      </c>
+    </row>
+    <row r="139" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A139" s="36">
         <v>59000</v>
       </c>
@@ -15033,6 +15372,9 @@
       </c>
       <c r="Q139" s="34">
         <v>0</v>
+      </c>
+      <c r="R139" s="36" t="s">
+        <v>230</v>
       </c>
     </row>
   </sheetData>

</xml_diff>